<commit_message>
updating lower san joaquin length
</commit_message>
<xml_diff>
--- a/data-raw/R2R_TMH_habitat_inputs/River Length Summary.xlsx
+++ b/data-raw/R2R_TMH_habitat_inputs/River Length Summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10409"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maddeerubenson/Documents/git/R2R/DSMhabitat/data-raw/R2R_TMH_habitat_inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563C7B9D-1D96-3F48-89DA-1FACFCC3E1C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCED162-C196-9A41-85D3-EF9615023BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32960" yWindow="2080" windowWidth="28800" windowHeight="15760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30200" yWindow="1520" windowWidth="34600" windowHeight="18580" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -29,9 +29,11 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -51,6 +53,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>@aidankelleher98@gmail.com what are the units here?
@@ -66,6 +69,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>@aidankelleher98@gmail.com need these values
@@ -91,6 +95,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>Table 2 of Yoshiyama; column 3
@@ -115,6 +120,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>not including Fall River, a tributary, which has an additional 24.3 mi</t>
@@ -128,6 +134,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>summing all subreach lengths</t>
@@ -141,6 +148,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>includes length of both reservoirs</t>
@@ -154,6 +162,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>including reach slightly downstream that is beyond the extent of the current habitat shapefile</t>
@@ -167,6 +176,7 @@
             <sz val="10"/>
             <color rgb="FF000000"/>
             <rFont val="Arial"/>
+            <family val="2"/>
             <scheme val="minor"/>
           </rPr>
           <t>including reach slightly downstream that is beyond the extent of the current habitat shapefile</t>
@@ -178,7 +188,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="728" uniqueCount="267">
   <si>
     <t>River lengths</t>
   </si>
@@ -756,9 +766,6 @@
     <t xml:space="preserve">To confluence with Merced River </t>
   </si>
   <si>
-    <t xml:space="preserve">Where does the SJ start?? </t>
-  </si>
-  <si>
     <t>North Delta</t>
   </si>
   <si>
@@ -981,6 +988,9 @@
   <si>
     <t>Friant Dam (Millerton Lake)</t>
   </si>
+  <si>
+    <t xml:space="preserve">SIT extent (Merced to South Delta) + Merced to Friant Dam </t>
+  </si>
 </sst>
 </file>
 
@@ -1002,6 +1012,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1009,12 +1020,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1022,11 +1035,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1037,12 +1052,14 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1054,12 +1071,14 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1067,6 +1086,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1074,6 +1094,7 @@
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -4871,7 +4892,7 @@
         <v>54</v>
       </c>
       <c r="F94" s="25">
-        <v>45</v>
+        <v>225.71090000000001</v>
       </c>
       <c r="G94" s="25"/>
       <c r="H94" s="25"/>
@@ -4879,11 +4900,9 @@
         <v>0</v>
       </c>
       <c r="J94" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="K94" s="25" t="s">
-        <v>192</v>
-      </c>
+        <v>266</v>
+      </c>
+      <c r="K94" s="25"/>
       <c r="L94" s="7" t="s">
         <v>185</v>
       </c>
@@ -4903,13 +4922,13 @@
     </row>
     <row r="95" spans="1:27" ht="16" x14ac:dyDescent="0.2">
       <c r="A95" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C95" s="25" t="s">
         <v>193</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="C95" s="25" t="s">
-        <v>194</v>
       </c>
       <c r="D95" s="25" t="s">
         <v>75</v>
@@ -4930,7 +4949,7 @@
       </c>
       <c r="K95" s="25"/>
       <c r="L95" s="7" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="M95" s="7" t="s">
         <v>77</v>
@@ -4946,13 +4965,13 @@
     </row>
     <row r="96" spans="1:27" ht="16" x14ac:dyDescent="0.2">
       <c r="A96" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C96" s="25" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D96" s="25" t="s">
         <v>75</v>
@@ -4973,7 +4992,7 @@
       </c>
       <c r="K96" s="25"/>
       <c r="L96" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M96" s="7" t="s">
         <v>77</v>
@@ -9836,7 +9855,7 @@
   <customSheetViews>
     <customSheetView guid="{82525D4F-3E41-4EA6-A509-DA05F63782D4}" filter="1" showAutoFilter="1">
       <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-      <autoFilter ref="A1:AA1061" xr:uid="{872D6F7C-064F-7E4B-9FF5-C230378D613F}">
+      <autoFilter ref="A1:AA1061" xr:uid="{942F7B0B-461E-2D44-8C60-9B980F87DD33}">
         <filterColumn colId="11">
           <filters>
             <filter val="USC"/>
@@ -9872,22 +9891,22 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="C1" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>202</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -9898,7 +9917,7 @@
         <v>28</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D2" s="1">
         <v>40682</v>
@@ -9917,10 +9936,10 @@
         <v>78</v>
       </c>
       <c r="B3" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>205</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="D3" s="1">
         <v>17723</v>
@@ -9930,7 +9949,7 @@
         <v>3.3566287878787877</v>
       </c>
       <c r="F3" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -9941,7 +9960,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D4" s="1">
         <v>25254</v>
@@ -9963,7 +9982,7 @@
         <v>52</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D5" s="1">
         <f>18.79*5280</f>
@@ -9986,7 +10005,7 @@
         <v>133</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D6" s="1">
         <v>39696</v>
@@ -10005,10 +10024,10 @@
         <v>67</v>
       </c>
       <c r="B7" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D7" s="1">
         <v>55617</v>
@@ -10018,7 +10037,7 @@
         <v>10.533522727272727</v>
       </c>
       <c r="F7" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10029,7 +10048,7 @@
         <v>147</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D8" s="1">
         <v>35097</v>
@@ -10048,10 +10067,10 @@
         <v>50</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D9" s="1">
         <v>44190</v>
@@ -10061,7 +10080,7 @@
         <v>8.3693181818181817</v>
       </c>
       <c r="F9" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10069,10 +10088,10 @@
         <v>50</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D10" s="1">
         <v>49831</v>
@@ -10082,7 +10101,7 @@
         <v>9.4376893939393938</v>
       </c>
       <c r="F10" s="28" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -10093,7 +10112,7 @@
         <v>56</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D11" s="1">
         <v>18572</v>
@@ -10115,7 +10134,7 @@
         <v>173</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D12" s="1">
         <v>44604</v>
@@ -10137,7 +10156,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D13" s="1">
         <v>11792</v>
@@ -10159,7 +10178,7 @@
         <v>66</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D14" s="1">
         <v>44921</v>
@@ -10181,7 +10200,7 @@
         <v>51</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D15" s="1">
         <v>18641</v>
@@ -10197,13 +10216,13 @@
     </row>
     <row r="16" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B16" s="28">
         <v>52</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D16" s="1">
         <f>E16*5280</f>
@@ -13192,7 +13211,7 @@
   <sheetData>
     <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A1" s="31" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -13223,7 +13242,7 @@
     </row>
     <row r="2" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="31" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B2" s="32"/>
       <c r="C2" s="32"/>
@@ -13283,28 +13302,28 @@
     </row>
     <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="32" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B4" s="32" t="s">
+        <v>222</v>
+      </c>
+      <c r="C4" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="C4" s="32" t="s">
+      <c r="D4" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="E4" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="D4" s="32" t="s">
-        <v>200</v>
-      </c>
-      <c r="E4" s="36" t="s">
+      <c r="F4" s="36" t="s">
         <v>225</v>
       </c>
-      <c r="F4" s="36" t="s">
+      <c r="G4" s="32" t="s">
         <v>226</v>
       </c>
-      <c r="G4" s="32" t="s">
+      <c r="H4" s="37" t="s">
         <v>227</v>
-      </c>
-      <c r="H4" s="37" t="s">
-        <v>228</v>
       </c>
       <c r="I4" s="35"/>
       <c r="J4" s="35"/>
@@ -13334,10 +13353,10 @@
         <v>51</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E5" s="40">
         <v>8</v>
@@ -13410,10 +13429,10 @@
         <v>9</v>
       </c>
       <c r="C7" s="38" t="s">
+        <v>228</v>
+      </c>
+      <c r="D7" s="38" t="s">
         <v>229</v>
-      </c>
-      <c r="D7" s="38" t="s">
-        <v>230</v>
       </c>
       <c r="E7" s="40">
         <v>9.5</v>
@@ -13480,11 +13499,11 @@
     </row>
     <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="38" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B9" s="28"/>
       <c r="C9" s="43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E9" s="44">
         <f t="shared" ref="E9:G9" si="0">E10+E11</f>
@@ -13525,10 +13544,10 @@
         <v>13</v>
       </c>
       <c r="C10" s="38" t="s">
+        <v>232</v>
+      </c>
+      <c r="D10" s="38" t="s">
         <v>233</v>
-      </c>
-      <c r="D10" s="38" t="s">
-        <v>234</v>
       </c>
       <c r="E10" s="40">
         <v>2.4</v>
@@ -13568,7 +13587,7 @@
       <c r="A11" s="38"/>
       <c r="B11" s="39"/>
       <c r="C11" s="46" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D11" s="38"/>
       <c r="E11" s="40">
@@ -13610,10 +13629,10 @@
         <v>52</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E12" s="40">
         <f>4.6+15.9</f>
@@ -13656,10 +13675,10 @@
         <v>50</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E13" s="40">
         <f>4.6+4.1+14.3</f>
@@ -13702,10 +13721,10 @@
         <v>99</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E14" s="40">
         <f>4.6+4.1+22.6</f>
@@ -13779,7 +13798,7 @@
         <v>147</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D16" s="38"/>
       <c r="E16" s="40">
@@ -13822,10 +13841,10 @@
       <c r="A17" s="38"/>
       <c r="B17" s="39"/>
       <c r="C17" s="38" t="s">
+        <v>238</v>
+      </c>
+      <c r="D17" s="38" t="s">
         <v>239</v>
-      </c>
-      <c r="D17" s="38" t="s">
-        <v>240</v>
       </c>
       <c r="E17" s="40">
         <f>2.1+7.5+8.7</f>
@@ -13863,10 +13882,10 @@
       <c r="A18" s="38"/>
       <c r="B18" s="39"/>
       <c r="C18" s="38" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E18" s="40">
         <f>2.1+7.5+12.3</f>
@@ -13905,10 +13924,10 @@
       <c r="A19" s="38"/>
       <c r="B19" s="39"/>
       <c r="C19" s="38" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E19" s="40">
         <f>2.1+2.8+12.5</f>
@@ -13946,10 +13965,10 @@
       <c r="A20" s="38"/>
       <c r="B20" s="39"/>
       <c r="C20" s="38" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D20" s="38" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E20" s="40">
         <f>2.1+2.8+8</f>
@@ -14020,7 +14039,7 @@
         <v>56</v>
       </c>
       <c r="C22" s="43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E22" s="47">
         <f t="shared" ref="E22:F22" si="4">SUM(E23:E24)</f>
@@ -14039,7 +14058,7 @@
         <v>49.899999999999991</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J22" s="38"/>
       <c r="K22" s="38"/>
@@ -14063,10 +14082,10 @@
     <row r="23" spans="1:27" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.15">
       <c r="A23" s="38"/>
       <c r="C23" s="38" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D23" s="38" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E23" s="40">
         <f>7.6+3.1+1.2</f>
@@ -14105,10 +14124,10 @@
       <c r="A24" s="38"/>
       <c r="B24" s="39"/>
       <c r="C24" s="38" t="s">
+        <v>245</v>
+      </c>
+      <c r="D24" s="38" t="s">
         <v>246</v>
-      </c>
-      <c r="D24" s="38" t="s">
-        <v>247</v>
       </c>
       <c r="E24" s="40">
         <v>15.4</v>
@@ -14178,7 +14197,7 @@
         <v>133</v>
       </c>
       <c r="C26" s="43" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E26" s="44">
         <f t="shared" ref="E26:G26" si="6">E27+E28</f>
@@ -14220,10 +14239,10 @@
       <c r="A27" s="38"/>
       <c r="B27" s="39"/>
       <c r="C27" s="38" t="s">
+        <v>247</v>
+      </c>
+      <c r="D27" s="38" t="s">
         <v>248</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>249</v>
       </c>
       <c r="E27" s="40">
         <v>7</v>
@@ -14260,7 +14279,7 @@
       <c r="A28" s="38"/>
       <c r="B28" s="39"/>
       <c r="C28" s="46" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D28" s="38"/>
       <c r="E28" s="40">
@@ -14300,10 +14319,10 @@
       <c r="A29" s="38"/>
       <c r="B29" s="39"/>
       <c r="C29" s="38" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D29" s="38" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E29" s="40">
         <f>0.7+11.5</f>
@@ -14341,10 +14360,10 @@
       <c r="A30" s="38"/>
       <c r="B30" s="39"/>
       <c r="C30" s="38" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D30" s="38" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="E30" s="40">
         <f>0.7+16.1</f>
@@ -14416,7 +14435,7 @@
         <v>28</v>
       </c>
       <c r="C32" s="43" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D32" s="38"/>
       <c r="E32" s="40">
@@ -14459,10 +14478,10 @@
       <c r="A33" s="38"/>
       <c r="B33" s="39"/>
       <c r="C33" s="38" t="s">
+        <v>253</v>
+      </c>
+      <c r="D33" s="38" t="s">
         <v>254</v>
-      </c>
-      <c r="D33" s="38" t="s">
-        <v>255</v>
       </c>
       <c r="E33" s="40">
         <v>10.6</v>
@@ -14499,10 +14518,10 @@
       <c r="A34" s="38"/>
       <c r="B34" s="39"/>
       <c r="C34" s="38" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D34" s="38" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E34" s="40">
         <v>7.3</v>
@@ -14573,7 +14592,7 @@
         <v>66</v>
       </c>
       <c r="C36" s="43" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E36" s="44">
         <f t="shared" ref="E36:G36" si="10">E37+E38</f>
@@ -14615,10 +14634,10 @@
       <c r="A37" s="38"/>
       <c r="B37" s="39"/>
       <c r="C37" s="38" t="s">
+        <v>256</v>
+      </c>
+      <c r="D37" s="38" t="s">
         <v>257</v>
-      </c>
-      <c r="D37" s="38" t="s">
-        <v>258</v>
       </c>
       <c r="E37" s="40">
         <v>10.3</v>
@@ -14655,10 +14674,10 @@
       <c r="A38" s="38"/>
       <c r="B38" s="39"/>
       <c r="C38" s="38" t="s">
+        <v>258</v>
+      </c>
+      <c r="D38" s="38" t="s">
         <v>259</v>
-      </c>
-      <c r="D38" s="38" t="s">
-        <v>260</v>
       </c>
       <c r="E38" s="40">
         <v>21.5</v>
@@ -14723,16 +14742,16 @@
     </row>
     <row r="40" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="38" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B40" s="39">
         <v>52</v>
       </c>
       <c r="C40" s="38" t="s">
+        <v>260</v>
+      </c>
+      <c r="D40" s="38" t="s">
         <v>261</v>
-      </c>
-      <c r="D40" s="38" t="s">
-        <v>262</v>
       </c>
       <c r="E40" s="40">
         <f>2.8+23.2</f>
@@ -14807,10 +14826,10 @@
         <v>56</v>
       </c>
       <c r="C42" s="38" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D42" s="38" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E42" s="40">
         <f>19.5+10.8</f>
@@ -14885,7 +14904,7 @@
         <v>173</v>
       </c>
       <c r="C44" s="43" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="E44" s="44">
         <f>E46</f>
@@ -14927,7 +14946,7 @@
       <c r="A45" s="38"/>
       <c r="B45" s="39"/>
       <c r="C45" s="38" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D45" s="38" t="s">
         <v>77</v>
@@ -14967,10 +14986,10 @@
       <c r="A46" s="38"/>
       <c r="B46" s="39"/>
       <c r="C46" s="38" t="s">
+        <v>264</v>
+      </c>
+      <c r="D46" s="38" t="s">
         <v>265</v>
-      </c>
-      <c r="D46" s="38" t="s">
-        <v>266</v>
       </c>
       <c r="E46" s="40">
         <v>14.8</v>

</xml_diff>